<commit_message>
Implementado Quadro de Ativos e Passivos Financeiros e Permanentes do BP e corrigido writer.
O writer da dcasp estava salvando apenas o último frame no xlsx.
</commit_message>
<xml_diff>
--- a/data/dcasp/2022/12/pm/bp.xlsx
+++ b/data/dcasp/2022/12/pm/bp.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="QuadroPrincipal" sheetId="1" r:id="rId1"/>
+    <sheet name="QuadroFinanceiroPermanente" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>Linha</t>
   </si>
@@ -25,7 +26,7 @@
     <t>ExercicioAnterior</t>
   </si>
   <si>
-    <t>AtivoTotal</t>
+    <t>Ativo</t>
   </si>
   <si>
     <t>AtivoCirculante</t>
@@ -35,6 +36,132 @@
   </si>
   <si>
     <t>CreditosACurtoPrazo</t>
+  </si>
+  <si>
+    <t>InvestimentosEAplicacoesTemporariasACurtoPrazo</t>
+  </si>
+  <si>
+    <t>Estoques</t>
+  </si>
+  <si>
+    <t>AtivoNaoCirculanteMantidoParaVenda</t>
+  </si>
+  <si>
+    <t>VPDPagasAntecipadamente</t>
+  </si>
+  <si>
+    <t>AtivoNaoCirculante</t>
+  </si>
+  <si>
+    <t>RealizavelALongoPrazo</t>
+  </si>
+  <si>
+    <t>Investimentos</t>
+  </si>
+  <si>
+    <t>Imobilizado</t>
+  </si>
+  <si>
+    <t>Intangivel</t>
+  </si>
+  <si>
+    <t>Diferido</t>
+  </si>
+  <si>
+    <t>PassivoEPatrimonioLiquido</t>
+  </si>
+  <si>
+    <t>PassivoCirculante</t>
+  </si>
+  <si>
+    <t>ObrigacoesTrabalhistasPrevidenciariasEAssistenciaisAPagarACurtoPrazo</t>
+  </si>
+  <si>
+    <t>EmprestimosEFinanciamentosACurtoPrazo</t>
+  </si>
+  <si>
+    <t>FornecedoresEContasAPagarACurtoPrazo</t>
+  </si>
+  <si>
+    <t>ObrigacoesFiscaisACurtoPrazo</t>
+  </si>
+  <si>
+    <t>ObrigacoesDeReparticoesAOutrosEntes</t>
+  </si>
+  <si>
+    <t>ProvisoesACurtoPrazo</t>
+  </si>
+  <si>
+    <t>DemaisObrigacoesACurtoPrazo</t>
+  </si>
+  <si>
+    <t>PassivoNaoCirculante</t>
+  </si>
+  <si>
+    <t>ObrigacoesTrabalhistasPrevidenciariasEAssistenciaisAPagarALongoPrazo</t>
+  </si>
+  <si>
+    <t>EmprestimosEFinanciamentosALongoPrazo</t>
+  </si>
+  <si>
+    <t>FornecedoresEContasAPagarALongoPrazo</t>
+  </si>
+  <si>
+    <t>ObrigacoesFiscaisALongoPrazo</t>
+  </si>
+  <si>
+    <t>ProvisoesALongoPrazo</t>
+  </si>
+  <si>
+    <t>DemaisObrigacoesALongoPrazo</t>
+  </si>
+  <si>
+    <t>ResultadoDiferido</t>
+  </si>
+  <si>
+    <t>PatrimonioLiquido</t>
+  </si>
+  <si>
+    <t>PatrimonioSocialECapitalSocial</t>
+  </si>
+  <si>
+    <t>AdiantamentoParaFuturoAumentoDeCapital</t>
+  </si>
+  <si>
+    <t>ReservasDeCapital</t>
+  </si>
+  <si>
+    <t>AjustesDeAvaliacaoPatrimonial</t>
+  </si>
+  <si>
+    <t>ReservasDeLucros</t>
+  </si>
+  <si>
+    <t>DemaisReservas</t>
+  </si>
+  <si>
+    <t>ResultadosAcumulados</t>
+  </si>
+  <si>
+    <t>AcoesCotasEmTesouraria</t>
+  </si>
+  <si>
+    <t>AtivoFinanceiro</t>
+  </si>
+  <si>
+    <t>AtivoPermanente</t>
+  </si>
+  <si>
+    <t>Passivo</t>
+  </si>
+  <si>
+    <t>PassivoFinanceiro</t>
+  </si>
+  <si>
+    <t>PassivoPermanente</t>
+  </si>
+  <si>
+    <t>SaldoPatrimonial</t>
   </si>
 </sst>
 </file>
@@ -392,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -450,6 +577,500 @@
         <v>762203.1</v>
       </c>
     </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>2885566.67</v>
+      </c>
+      <c r="C7">
+        <v>3243749.73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>271070.47</v>
+      </c>
+      <c r="C8">
+        <v>271070.47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>83494</v>
+      </c>
+      <c r="C9">
+        <v>120620.66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10">
+        <v>18544464.66</v>
+      </c>
+      <c r="C10">
+        <v>20870475.57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>8955.729999999981</v>
+      </c>
+      <c r="C11">
+        <v>3988.309999999935</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12">
+        <v>97076.16</v>
+      </c>
+      <c r="C12">
+        <v>167007.36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>18438432.77</v>
+      </c>
+      <c r="C13">
+        <v>20699479.9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <v>29259587.85999999</v>
+      </c>
+      <c r="C16">
+        <v>32091749.87999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17">
+        <v>609238.9400000001</v>
+      </c>
+      <c r="C17">
+        <v>629313.3200000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18">
+        <v>537981.17</v>
+      </c>
+      <c r="C18">
+        <v>518836.23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20">
+        <v>40444.9</v>
+      </c>
+      <c r="C20">
+        <v>52086.31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21">
+        <v>30812.87</v>
+      </c>
+      <c r="C21">
+        <v>30172.9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>28217.88</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25">
+        <v>3849430.23</v>
+      </c>
+      <c r="C25">
+        <v>4270773.43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26">
+        <v>1822914.66</v>
+      </c>
+      <c r="C26">
+        <v>1987381.87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30">
+        <v>2026515.57</v>
+      </c>
+      <c r="C30">
+        <v>2283391.56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33">
+        <v>24800918.68999999</v>
+      </c>
+      <c r="C33">
+        <v>27191663.12999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40">
+        <v>24800918.68999999</v>
+      </c>
+      <c r="C40">
+        <v>27191663.12999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41">
+        <v>0</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>29259587.86</v>
+      </c>
+      <c r="C2">
+        <v>32091749.88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3">
+        <v>7238339.869999999</v>
+      </c>
+      <c r="C3">
+        <v>6823912.699999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4">
+        <v>22021247.99</v>
+      </c>
+      <c r="C4">
+        <v>25267837.18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5">
+        <v>4458669.17</v>
+      </c>
+      <c r="C5">
+        <v>4900086.75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6">
+        <v>63681.14999999999</v>
+      </c>
+      <c r="C6">
+        <v>420159.04</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7">
+        <v>4397388.02</v>
+      </c>
+      <c r="C7">
+        <v>4740581</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8">
+        <v>27191663.13</v>
+      </c>
+      <c r="C8">
+        <v>24800918.69000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Adicionados novos quadros no dcasp/bp.
</commit_message>
<xml_diff>
--- a/data/dcasp/2022/12/pm/bp.xlsx
+++ b/data/dcasp/2022/12/pm/bp.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="QuadroPrincipal" sheetId="1" r:id="rId1"/>
     <sheet name="QuadroFinanceiroPermanente" sheetId="2" r:id="rId2"/>
+    <sheet name="QuadroCompensacao" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
   <si>
     <t>Linha</t>
   </si>
@@ -162,6 +163,36 @@
   </si>
   <si>
     <t>SaldoPatrimonial</t>
+  </si>
+  <si>
+    <t>AtosPotenciaisAtivos</t>
+  </si>
+  <si>
+    <t>GarantiasEContragarantiasRecebidas</t>
+  </si>
+  <si>
+    <t>DireitosConveniadosEOutrosInstrumentosCongeneres</t>
+  </si>
+  <si>
+    <t>DireitosContratuais</t>
+  </si>
+  <si>
+    <t>OutrosAtosPotenciaisAtivos</t>
+  </si>
+  <si>
+    <t>AtosPotenciaisPassivos</t>
+  </si>
+  <si>
+    <t>GarantiasEContragarantiasConcedidas</t>
+  </si>
+  <si>
+    <t>ObrigacoesConveniadasEOutrosInstrumentosCongeneres</t>
+  </si>
+  <si>
+    <t>ObrigacoesContratuais</t>
+  </si>
+  <si>
+    <t>OutrosAtosPotenciaisPassivos</t>
   </si>
 </sst>
 </file>
@@ -1074,4 +1105,135 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2">
+        <v>218238.07</v>
+      </c>
+      <c r="C2">
+        <v>220672.22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5">
+        <v>17414</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6">
+        <v>200824.07</v>
+      </c>
+      <c r="C6">
+        <v>220672.22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7">
+        <v>3737173.3</v>
+      </c>
+      <c r="C7">
+        <v>9825079.249999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9">
+        <v>63270</v>
+      </c>
+      <c r="C9">
+        <v>78586.62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10">
+        <v>3464390.71</v>
+      </c>
+      <c r="C10">
+        <v>9617552.629999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11">
+        <v>209512.59</v>
+      </c>
+      <c r="C11">
+        <v>128940</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>